<commit_message>
Atualiza documentos de referencia com as mudancas recentes do site
- inventario-de-conteudo.xlsx: corrige maiuscula das especialidades,
  remove linha da citacao removida de artigo.html, reordena cards de
  especialidade (Home e hub) e condicoes de Dermatologia
- relatorio-alt-title-imagens.xlsx: mesma reordenacao de imagens/icones
- documentacao-componentes.pdf: documenta a nova faixa de breakpoint
  de tablet (721-1024px) e a ordem atual de SPECIALTY_CONDITIONS

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/relatorio-alt-title-imagens.xlsx
+++ b/relatorio-alt-title-imagens.xlsx
@@ -1082,17 +1082,17 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>assets/images/specialty-cardiologia.png</t>
+          <t>assets/images/specialty-dermatologia.png</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>Homem e mulher sêniores abraçados e rindo em uma área arborizada ao pôr do sol.</t>
+          <t>Homem de cabelo afro sorrindo para a câmera em uma área externa, com outra pessoa ao fundo.</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>Casal idoso abraçado e sorrindo ao ar livre</t>
+          <t>Homem sorridente em área externa</t>
         </is>
       </c>
     </row>
@@ -1107,17 +1107,17 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>assets/images/specialty-dermatologia.png</t>
+          <t>assets/images/specialty-oncologia.png</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>Homem de cabelo afro sorrindo para a câmera em uma área externa, com outra pessoa ao fundo.</t>
+          <t>Mulher de camiseta roxa com os braços abertos olhando para cima durante aula de yoga ao ar livre.</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>Homem sorridente em área externa</t>
+          <t>Prática de yoga ao ar livre em grupo</t>
         </is>
       </c>
     </row>
@@ -1132,17 +1132,17 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>assets/images/specialty-hematologia.png</t>
+          <t>assets/images/specialty-neurologia.png</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>Homem de dreadlocks e mulher sorridente sentados na areia da praia, brindando com garrafas de bebida sob a luz do sol.</t>
+          <t>Mulher idosa segurando um bebê no ar com carinho no jardim em frente a uma casa.</t>
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>Casal brindando com bebidas em dia ensolarado na praia</t>
+          <t>Avó segurando bebê ao ar livre</t>
         </is>
       </c>
     </row>
@@ -1157,17 +1157,17 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>assets/images/specialty-nefrologia.png</t>
+          <t>assets/images/specialty-cardiologia.png</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>Avô, mãe e garotinho sentados juntos em um sofá na sala de estar, interagindo alegremente.</t>
+          <t>Homem e mulher sêniores abraçados e rindo em uma área arborizada ao pôr do sol.</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>Família reunida sorrindo no sofá de casa</t>
+          <t>Casal idoso abraçado e sorrindo ao ar livre</t>
         </is>
       </c>
     </row>
@@ -1182,17 +1182,17 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>assets/images/specialty-neurologia.png</t>
+          <t>assets/images/specialty-hematologia.png</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>Mulher idosa segurando um bebê no ar com carinho no jardim em frente a uma casa.</t>
+          <t>Homem de dreadlocks e mulher sorridente sentados na areia da praia, brindando com garrafas de bebida sob a luz do sol.</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>Avó segurando bebê ao ar livre</t>
+          <t>Casal brindando com bebidas em dia ensolarado na praia</t>
         </is>
       </c>
     </row>
@@ -1207,17 +1207,17 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>assets/images/specialty-oncologia.png</t>
+          <t>assets/images/specialty-nefrologia.png</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>Mulher de camiseta roxa com os braços abertos olhando para cima durante aula de yoga ao ar livre.</t>
+          <t>Avô, mãe e garotinho sentados juntos em um sofá na sala de estar, interagindo alegremente.</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>Prática de yoga ao ar livre em grupo</t>
+          <t>Família reunida sorrindo no sofá de casa</t>
         </is>
       </c>
     </row>
@@ -9269,7 +9269,7 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>../assets/icons/condition-urticaria.svg</t>
+          <t>../assets/icons/condition-psoriase.svg</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
@@ -9290,7 +9290,7 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>../assets/icons/condition-psoriase.svg</t>
+          <t>../assets/icons/condition-urticaria.svg</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
@@ -21541,7 +21541,7 @@
           <t>(vazio)</t>
         </is>
       </c>
-      <c r="E23" s="3" t="inlineStr"/>
+      <c r="E23" s="3" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
@@ -21554,7 +21554,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>../assets/icons/condition-infarto.svg</t>
+          <t>../assets/icons/condition-hidradenite-supurativa.svg</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
@@ -21562,7 +21562,7 @@
           <t>(vazio)</t>
         </is>
       </c>
-      <c r="E24" s="3" t="inlineStr"/>
+      <c r="E24" s="3" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
@@ -21575,7 +21575,7 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>../assets/icons/condition-colesterol-alto.svg</t>
+          <t>../assets/icons/condition-furunculo.svg</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
@@ -21583,7 +21583,7 @@
           <t>(vazio)</t>
         </is>
       </c>
-      <c r="E25" s="3" t="inlineStr"/>
+      <c r="E25" s="3" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
@@ -21596,7 +21596,7 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>../assets/icons/accordion-chevron.svg</t>
+          <t>../assets/icons/condition-psoriase.svg</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
@@ -21604,7 +21604,7 @@
           <t>(vazio)</t>
         </is>
       </c>
-      <c r="E26" s="3" t="inlineStr"/>
+      <c r="E26" s="3" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
@@ -21617,7 +21617,7 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>../assets/icons/condition-hidradenite-supurativa.svg</t>
+          <t>../assets/icons/condition-urticaria.svg</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
@@ -21625,7 +21625,7 @@
           <t>(vazio)</t>
         </is>
       </c>
-      <c r="E27" s="3" t="inlineStr"/>
+      <c r="E27" s="3" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
@@ -21638,7 +21638,7 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>../assets/icons/condition-furunculo.svg</t>
+          <t>../assets/icons/accordion-chevron.svg</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
@@ -21646,7 +21646,7 @@
           <t>(vazio)</t>
         </is>
       </c>
-      <c r="E28" s="3" t="inlineStr"/>
+      <c r="E28" s="3" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
@@ -21659,7 +21659,7 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>../assets/icons/condition-urticaria.svg</t>
+          <t>../assets/icons/condition-cancer-mama.svg</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
@@ -21667,7 +21667,7 @@
           <t>(vazio)</t>
         </is>
       </c>
-      <c r="E29" s="3" t="inlineStr"/>
+      <c r="E29" s="3" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
@@ -21680,7 +21680,7 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>../assets/icons/condition-psoriase.svg</t>
+          <t>../assets/icons/condition-cancer-prostata.svg</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
@@ -21688,7 +21688,7 @@
           <t>(vazio)</t>
         </is>
       </c>
-      <c r="E30" s="3" t="inlineStr"/>
+      <c r="E30" s="3" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
@@ -21709,7 +21709,7 @@
           <t>(vazio)</t>
         </is>
       </c>
-      <c r="E31" s="3" t="inlineStr"/>
+      <c r="E31" s="3" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
@@ -21722,7 +21722,7 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>../assets/icons/condition-hpn.svg</t>
+          <t>../assets/icons/condition-esclerose-multipla.svg</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
@@ -21730,7 +21730,7 @@
           <t>(vazio)</t>
         </is>
       </c>
-      <c r="E32" s="3" t="inlineStr"/>
+      <c r="E32" s="3" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
@@ -21743,7 +21743,7 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>../assets/icons/condition-lmc.svg</t>
+          <t>../assets/icons/condition-ame.svg</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
@@ -21751,7 +21751,7 @@
           <t>(vazio)</t>
         </is>
       </c>
-      <c r="E33" s="3" t="inlineStr"/>
+      <c r="E33" s="3" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
@@ -21764,7 +21764,7 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>../assets/icons/condition-mielofibrose.svg</t>
+          <t>../assets/icons/accordion-chevron.svg</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
@@ -21772,7 +21772,7 @@
           <t>(vazio)</t>
         </is>
       </c>
-      <c r="E34" s="3" t="inlineStr"/>
+      <c r="E34" s="3" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
@@ -21785,7 +21785,7 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>../assets/icons/accordion-chevron.svg</t>
+          <t>../assets/icons/condition-infarto.svg</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
@@ -21793,7 +21793,7 @@
           <t>(vazio)</t>
         </is>
       </c>
-      <c r="E35" s="3" t="inlineStr"/>
+      <c r="E35" s="3" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
@@ -21806,7 +21806,7 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>../assets/icons/condition-doencas-renais-graves.svg</t>
+          <t>../assets/icons/condition-colesterol-alto.svg</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
@@ -21814,7 +21814,7 @@
           <t>(vazio)</t>
         </is>
       </c>
-      <c r="E36" s="3" t="inlineStr"/>
+      <c r="E36" s="3" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
@@ -21835,7 +21835,7 @@
           <t>(vazio)</t>
         </is>
       </c>
-      <c r="E37" s="3" t="inlineStr"/>
+      <c r="E37" s="3" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
@@ -21848,7 +21848,7 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>../assets/icons/condition-esclerose-multipla.svg</t>
+          <t>../assets/icons/condition-hpn.svg</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
@@ -21856,7 +21856,7 @@
           <t>(vazio)</t>
         </is>
       </c>
-      <c r="E38" s="3" t="inlineStr"/>
+      <c r="E38" s="3" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
@@ -21869,7 +21869,7 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>../assets/icons/condition-ame.svg</t>
+          <t>../assets/icons/condition-lmc.svg</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
@@ -21877,7 +21877,7 @@
           <t>(vazio)</t>
         </is>
       </c>
-      <c r="E39" s="3" t="inlineStr"/>
+      <c r="E39" s="3" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
@@ -21890,7 +21890,7 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>../assets/icons/accordion-chevron.svg</t>
+          <t>../assets/icons/condition-mielofibrose.svg</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
@@ -21898,7 +21898,7 @@
           <t>(vazio)</t>
         </is>
       </c>
-      <c r="E40" s="3" t="inlineStr"/>
+      <c r="E40" s="3" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
@@ -21911,7 +21911,7 @@
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>../assets/icons/condition-cancer-mama.svg</t>
+          <t>../assets/icons/accordion-chevron.svg</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
@@ -21919,7 +21919,7 @@
           <t>(vazio)</t>
         </is>
       </c>
-      <c r="E41" s="3" t="inlineStr"/>
+      <c r="E41" s="3" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
@@ -21932,7 +21932,7 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>../assets/icons/condition-cancer-prostata.svg</t>
+          <t>../assets/icons/condition-doencas-renais-graves.svg</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
@@ -21940,7 +21940,7 @@
           <t>(vazio)</t>
         </is>
       </c>
-      <c r="E42" s="3" t="inlineStr"/>
+      <c r="E42" s="3" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
@@ -21961,7 +21961,7 @@
           <t>(vazio)</t>
         </is>
       </c>
-      <c r="E43" s="3" t="inlineStr"/>
+      <c r="E43" s="3" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
@@ -21982,7 +21982,7 @@
           <t>(vazio)</t>
         </is>
       </c>
-      <c r="E44" s="3" t="inlineStr"/>
+      <c r="E44" s="3" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
@@ -22003,7 +22003,7 @@
           <t>(vazio)</t>
         </is>
       </c>
-      <c r="E45" s="3" t="inlineStr"/>
+      <c r="E45" s="3" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
@@ -22024,7 +22024,7 @@
           <t>(vazio)</t>
         </is>
       </c>
-      <c r="E46" s="3" t="inlineStr"/>
+      <c r="E46" s="3" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
@@ -22045,7 +22045,7 @@
           <t>(vazio)</t>
         </is>
       </c>
-      <c r="E47" s="3" t="inlineStr"/>
+      <c r="E47" s="3" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">

</xml_diff>